<commit_message>
Import existing Hire/Standby/No Hire status from the workbook and drop the Suggested column
Co-authored-by: konyebin <konyebin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/candidate-tracker/samples/FY27Q3_AMER_ASE_Scores_TEST_DATA.xlsx
+++ b/candidate-tracker/samples/FY27Q3_AMER_ASE_Scores_TEST_DATA.xlsx
@@ -1475,7 +1475,11 @@
         <f>Y11/48</f>
         <v/>
       </c>
-      <c r="AA11" s="34" t="n"/>
+      <c r="AA11" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB11" s="34" t="n"/>
       <c r="AC11" s="39" t="n"/>
     </row>
@@ -1581,7 +1585,11 @@
         <f>Y12/48</f>
         <v/>
       </c>
-      <c r="AA12" s="34" t="n"/>
+      <c r="AA12" s="34" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
       <c r="AB12" s="34" t="inlineStr">
         <is>
           <t>P. Morales</t>
@@ -1691,7 +1699,11 @@
         <f>Y13/48</f>
         <v/>
       </c>
-      <c r="AA13" s="34" t="n"/>
+      <c r="AA13" s="34" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
       <c r="AB13" s="34" t="inlineStr">
         <is>
           <t>P. Morales</t>
@@ -1801,7 +1813,11 @@
         <f>Y14/48</f>
         <v/>
       </c>
-      <c r="AA14" s="34" t="n"/>
+      <c r="AA14" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB14" s="34" t="n"/>
       <c r="AC14" s="39" t="n"/>
     </row>
@@ -1907,7 +1923,11 @@
         <f>Y15/48</f>
         <v/>
       </c>
-      <c r="AA15" s="34" t="n"/>
+      <c r="AA15" s="34" t="inlineStr">
+        <is>
+          <t>No Hire</t>
+        </is>
+      </c>
       <c r="AB15" s="34" t="n"/>
       <c r="AC15" s="39" t="n"/>
     </row>
@@ -2123,7 +2143,11 @@
         <f>Y17/48</f>
         <v/>
       </c>
-      <c r="AA17" s="34" t="n"/>
+      <c r="AA17" s="34" t="inlineStr">
+        <is>
+          <t>No Hire</t>
+        </is>
+      </c>
       <c r="AB17" s="34" t="n"/>
       <c r="AC17" s="39" t="n"/>
     </row>
@@ -2229,7 +2253,11 @@
         <f>Y18/48</f>
         <v/>
       </c>
-      <c r="AA18" s="34" t="n"/>
+      <c r="AA18" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB18" s="34" t="n"/>
       <c r="AC18" s="39" t="n"/>
     </row>
@@ -2335,7 +2363,11 @@
         <f>Y19/48</f>
         <v/>
       </c>
-      <c r="AA19" s="34" t="n"/>
+      <c r="AA19" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB19" s="34" t="n"/>
       <c r="AC19" s="39" t="n"/>
     </row>
@@ -2441,7 +2473,11 @@
         <f>Y20/48</f>
         <v/>
       </c>
-      <c r="AA20" s="34" t="n"/>
+      <c r="AA20" s="34" t="inlineStr">
+        <is>
+          <t>Hire</t>
+        </is>
+      </c>
       <c r="AB20" s="34" t="inlineStr">
         <is>
           <t>P. Morales</t>
@@ -2551,7 +2587,11 @@
         <f>Y21/48</f>
         <v/>
       </c>
-      <c r="AA21" s="34" t="n"/>
+      <c r="AA21" s="34" t="inlineStr">
+        <is>
+          <t>No Hire</t>
+        </is>
+      </c>
       <c r="AB21" s="34" t="n"/>
       <c r="AC21" s="39" t="n"/>
     </row>
@@ -2767,7 +2807,11 @@
         <f>Y23/48</f>
         <v/>
       </c>
-      <c r="AA23" s="34" t="n"/>
+      <c r="AA23" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB23" s="34" t="n"/>
       <c r="AC23" s="39" t="n"/>
     </row>
@@ -2873,7 +2917,11 @@
         <f>Y24/48</f>
         <v/>
       </c>
-      <c r="AA24" s="34" t="n"/>
+      <c r="AA24" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB24" s="34" t="n"/>
       <c r="AC24" s="39" t="n"/>
     </row>
@@ -2979,7 +3027,11 @@
         <f>Y25/48</f>
         <v/>
       </c>
-      <c r="AA25" s="34" t="n"/>
+      <c r="AA25" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB25" s="34" t="n"/>
       <c r="AC25" s="39" t="n"/>
     </row>
@@ -3085,7 +3137,11 @@
         <f>Y26/48</f>
         <v/>
       </c>
-      <c r="AA26" s="34" t="n"/>
+      <c r="AA26" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB26" s="34" t="n"/>
       <c r="AC26" s="39" t="n"/>
     </row>
@@ -3191,7 +3247,11 @@
         <f>Y27/48</f>
         <v/>
       </c>
-      <c r="AA27" s="34" t="n"/>
+      <c r="AA27" s="34" t="inlineStr">
+        <is>
+          <t>No Hire</t>
+        </is>
+      </c>
       <c r="AB27" s="34" t="n"/>
       <c r="AC27" s="39" t="n"/>
     </row>
@@ -3407,7 +3467,11 @@
         <f>Y29/48</f>
         <v/>
       </c>
-      <c r="AA29" s="34" t="n"/>
+      <c r="AA29" s="34" t="inlineStr">
+        <is>
+          <t>No Hire</t>
+        </is>
+      </c>
       <c r="AB29" s="34" t="n"/>
       <c r="AC29" s="39" t="n"/>
     </row>
@@ -3497,7 +3561,11 @@
         <f>Y30/48</f>
         <v/>
       </c>
-      <c r="AA30" s="34" t="n"/>
+      <c r="AA30" s="34" t="inlineStr">
+        <is>
+          <t>Standby</t>
+        </is>
+      </c>
       <c r="AB30" s="34" t="n"/>
       <c r="AC30" s="39" t="n"/>
     </row>

</xml_diff>